<commit_message>
adjusted testing scenarios to reflect fixes
</commit_message>
<xml_diff>
--- a/rules/CORE-001080/positive/03/data/unit-test-coreid-CG0288-positive3.xlsx
+++ b/rules/CORE-001080/positive/03/data/unit-test-coreid-CG0288-positive3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian_try2\core-contributor\rules\CORE-001080\positive\03\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\CORE-001080\positive\03\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92E96F3A-9853-4F5D-8F0A-43B33B762BBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EA0CB2B-9419-45A5-BB34-5AAE065C0323}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="361" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="361" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="91" r:id="rId1"/>
@@ -226,9 +226,6 @@
     <t>sdtmct</t>
   </si>
   <si>
-    <t>2016-09-30</t>
-  </si>
-  <si>
     <t>2016-06-24</t>
   </si>
   <si>
@@ -239,6 +236,9 @@
   </si>
   <si>
     <t>Culture Medium Type</t>
+  </si>
+  <si>
+    <t>2024-09-27</t>
   </si>
 </sst>
 </file>
@@ -311,7 +311,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -322,10 +322,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -954,23 +950,23 @@
       <c r="C6" s="2">
         <v>1</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I6" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="J6" s="6" t="s">
+      <c r="I6" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="K6" s="7" t="s">
-        <v>63</v>
+      <c r="K6" s="5" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -1171,6 +1167,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Comment xmlns="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010090ADB40D834AE945B19FCDA4041AC0CB" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d36826f407302d9fd93d8089214679b0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xmlns:ns3="63ea592b-d684-45c7-8cdc-fad8f8e6bb41" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="257daeb82d9c284d9d656fb5e9ad601e" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1410,26 +1425,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F04EB3C1-E279-4752-95AF-A2254F34364B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Comment xmlns="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF9BEA20-DCD2-4199-AEB6-4F95B371C878}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90113CEE-35A4-4503-9D90-53C6490D5D89}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1447,23 +1462,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF9BEA20-DCD2-4199-AEB6-4F95B371C878}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F04EB3C1-E279-4752-95AF-A2254F34364B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>